<commit_message>
MAJ carnet risques et obstacles Sprint 2
</commit_message>
<xml_diff>
--- a/docs/TP2-FoxTrot-Liste_Activites-Sprint2.xlsx
+++ b/docs/TP2-FoxTrot-Liste_Activites-Sprint2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UQAM\Été 2026\INF6150 (Génie logiciel - Conduite de projets informatiques)\Travaux Pratiques\TP2\fixmycar\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C25FA279-3CD5-4353-944F-A0A85A8DECAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29221729-89D3-48F5-BB5A-E3BCDFE2995D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Activités" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="149">
   <si>
     <t>Liste d'activités</t>
   </si>
@@ -519,6 +519,24 @@
   </si>
   <si>
     <t>Champs texte provisoires en attendant les FK définitives</t>
+  </si>
+  <si>
+    <t>Migration Django incompatible</t>
+  </si>
+  <si>
+    <t>Après ajout de AUTH_USER_MODEL, la base de données existante était incompatible — nécessitait de supprimer db.sqlite3 et refaire les migrations</t>
+  </si>
+  <si>
+    <t>Suppression de db.sqlite3 et relance de migrate pour recréer la base proprement</t>
+  </si>
+  <si>
+    <t>Module django_filters manquant</t>
+  </si>
+  <si>
+    <t>Après git pull, l'app vehicules de GAM nécessitait django-filter non installé localement</t>
+  </si>
+  <si>
+    <t>Installation via pip install django-filter dans l'environnement virtuel</t>
   </si>
 </sst>
 </file>
@@ -1781,6 +1799,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="16" fontId="16" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1837,9 +1858,6 @@
     </xf>
     <xf numFmtId="16" fontId="17" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1882,6 +1900,150 @@
           <bgColor theme="5"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2081,150 +2243,6 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -2253,35 +2271,35 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3A12FB0F-C40A-B748-8030-98D340CFAB34}" name="Tableau2" displayName="Tableau2" ref="A4:G10" totalsRowShown="0" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3A12FB0F-C40A-B748-8030-98D340CFAB34}" name="Tableau2" displayName="Tableau2" ref="A4:G10" totalsRowShown="0" dataDxfId="11">
   <autoFilter ref="A4:G10" xr:uid="{8AE4CE81-0313-2046-8C9D-FC8A5BDAF35E}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{36580D9E-E44F-E144-9187-9D6816E7AD65}" name="No." dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{EF559DC7-F47B-9848-8130-B462D7345CF6}" name="Titre court" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{82194528-C6CF-814C-9068-B4CEE7AB8C8E}" name="Description" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{FD6B68BF-B7A7-6B4C-89C4-B008807F3FC2}" name="Date de création" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{9BF3BF16-17B1-F146-97D3-9D22567C832F}" name="Affecté à (initiales)" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{7AF9C5EC-5B6E-5C43-B14B-1BBD1D028344}" name="Statut" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{A53E42DA-438D-C749-AC68-3D736120C878}" name="Solution envisagée ou appliquée" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{36580D9E-E44F-E144-9187-9D6816E7AD65}" name="No." dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{EF559DC7-F47B-9848-8130-B462D7345CF6}" name="Titre court" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{82194528-C6CF-814C-9068-B4CEE7AB8C8E}" name="Description" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{FD6B68BF-B7A7-6B4C-89C4-B008807F3FC2}" name="Date de création" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{9BF3BF16-17B1-F146-97D3-9D22567C832F}" name="Affecté à (initiales)" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{7AF9C5EC-5B6E-5C43-B14B-1BBD1D028344}" name="Statut" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{A53E42DA-438D-C749-AC68-3D736120C878}" name="Solution envisagée ou appliquée" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B8EC000B-D60C-D54E-89A3-4DAFB6D317CF}" name="Tableau3" displayName="Tableau3" ref="A4:J9" totalsRowShown="0" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B8EC000B-D60C-D54E-89A3-4DAFB6D317CF}" name="Tableau3" displayName="Tableau3" ref="A4:J9" totalsRowShown="0" dataDxfId="22">
   <autoFilter ref="A4:J9" xr:uid="{E1E6DC87-7A9F-264E-BA03-CD93728E459B}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{700F170B-9E35-454D-B601-2C8F61AC472A}" name="No." dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{69AD1862-3369-2F48-9B47-23217AD6E1A7}" name="Titre court" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{1204722B-3D6B-0843-9A2E-7ED16DAED71A}" name="Description du risque" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{6CE70BC6-06C1-D24D-98D7-4A3E45D6488D}" name="Probabilité d'occurrence" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{C1803549-A0D1-3B45-A312-78E45EC1161F}" name="Niveau d'impact" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{AB57BB6B-52E7-7147-B89C-61E7504410DB}" name="Date de création" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{4A075D44-5451-5A41-8EB6-CFDC70386649}" name="Affecté à (initiales)" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{32D938AC-3C43-104A-96A5-6759770A9983}" name="Statut" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{9C3D641B-166E-7A4F-8FEA-A4067A23B751}" name="Plan(s) de mitigation" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{43F9D95D-A1C9-D540-AD50-99C65F9EF0BB}" name="Plan(s) de contingence" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{700F170B-9E35-454D-B601-2C8F61AC472A}" name="No." dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{69AD1862-3369-2F48-9B47-23217AD6E1A7}" name="Titre court" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{1204722B-3D6B-0843-9A2E-7ED16DAED71A}" name="Description du risque" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{6CE70BC6-06C1-D24D-98D7-4A3E45D6488D}" name="Probabilité d'occurrence" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{C1803549-A0D1-3B45-A312-78E45EC1161F}" name="Niveau d'impact" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{AB57BB6B-52E7-7147-B89C-61E7504410DB}" name="Date de création" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{4A075D44-5451-5A41-8EB6-CFDC70386649}" name="Affecté à (initiales)" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{32D938AC-3C43-104A-96A5-6759770A9983}" name="Statut" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{9C3D641B-166E-7A4F-8FEA-A4067A23B751}" name="Plan(s) de mitigation" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{43F9D95D-A1C9-D540-AD50-99C65F9EF0BB}" name="Plan(s) de contingence" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2538,120 +2556,120 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="209" t="s">
+      <c r="B1" s="210" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="209"/>
-      <c r="D1" s="209"/>
-      <c r="E1" s="209"/>
-      <c r="F1" s="209"/>
-      <c r="G1" s="209"/>
-      <c r="H1" s="209"/>
-      <c r="I1" s="209"/>
-      <c r="J1" s="209"/>
-      <c r="K1" s="209"/>
+      <c r="C1" s="210"/>
+      <c r="D1" s="210"/>
+      <c r="E1" s="210"/>
+      <c r="F1" s="210"/>
+      <c r="G1" s="210"/>
+      <c r="H1" s="210"/>
+      <c r="I1" s="210"/>
+      <c r="J1" s="210"/>
+      <c r="K1" s="210"/>
       <c r="L1" s="11"/>
-      <c r="M1" s="211" t="s">
+      <c r="M1" s="212" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="211"/>
-      <c r="O1" s="211"/>
-      <c r="P1" s="211"/>
-      <c r="Q1" s="211"/>
-      <c r="R1" s="211"/>
-      <c r="S1" s="211"/>
-      <c r="T1" s="211"/>
-      <c r="U1" s="211"/>
-      <c r="V1" s="211"/>
-      <c r="W1" s="211"/>
-      <c r="X1" s="211"/>
-      <c r="Y1" s="211"/>
-      <c r="Z1" s="211"/>
-      <c r="AA1" s="211"/>
-      <c r="AB1" s="211"/>
-      <c r="AC1" s="211"/>
+      <c r="N1" s="212"/>
+      <c r="O1" s="212"/>
+      <c r="P1" s="212"/>
+      <c r="Q1" s="212"/>
+      <c r="R1" s="212"/>
+      <c r="S1" s="212"/>
+      <c r="T1" s="212"/>
+      <c r="U1" s="212"/>
+      <c r="V1" s="212"/>
+      <c r="W1" s="212"/>
+      <c r="X1" s="212"/>
+      <c r="Y1" s="212"/>
+      <c r="Z1" s="212"/>
+      <c r="AA1" s="212"/>
+      <c r="AB1" s="212"/>
+      <c r="AC1" s="212"/>
     </row>
     <row r="2" spans="1:43" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="203" t="s">
+      <c r="B2" s="204" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="203"/>
-      <c r="D2" s="203"/>
-      <c r="E2" s="203"/>
-      <c r="F2" s="203"/>
-      <c r="G2" s="203"/>
-      <c r="H2" s="203"/>
-      <c r="I2" s="203"/>
-      <c r="J2" s="203"/>
-      <c r="K2" s="203"/>
+      <c r="C2" s="204"/>
+      <c r="D2" s="204"/>
+      <c r="E2" s="204"/>
+      <c r="F2" s="204"/>
+      <c r="G2" s="204"/>
+      <c r="H2" s="204"/>
+      <c r="I2" s="204"/>
+      <c r="J2" s="204"/>
+      <c r="K2" s="204"/>
       <c r="L2" s="54"/>
-      <c r="M2" s="210" t="s">
+      <c r="M2" s="211" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="210"/>
-      <c r="O2" s="210"/>
-      <c r="P2" s="210"/>
-      <c r="Q2" s="210"/>
-      <c r="R2" s="210"/>
-      <c r="S2" s="210"/>
-      <c r="T2" s="210"/>
-      <c r="U2" s="210"/>
-      <c r="V2" s="210"/>
-      <c r="W2" s="210"/>
-      <c r="X2" s="210"/>
-      <c r="Y2" s="210"/>
-      <c r="Z2" s="210"/>
-      <c r="AA2" s="210"/>
-      <c r="AB2" s="210"/>
-      <c r="AC2" s="210"/>
+      <c r="N2" s="211"/>
+      <c r="O2" s="211"/>
+      <c r="P2" s="211"/>
+      <c r="Q2" s="211"/>
+      <c r="R2" s="211"/>
+      <c r="S2" s="211"/>
+      <c r="T2" s="211"/>
+      <c r="U2" s="211"/>
+      <c r="V2" s="211"/>
+      <c r="W2" s="211"/>
+      <c r="X2" s="211"/>
+      <c r="Y2" s="211"/>
+      <c r="Z2" s="211"/>
+      <c r="AA2" s="211"/>
+      <c r="AB2" s="211"/>
+      <c r="AC2" s="211"/>
       <c r="AF2" s="148"/>
       <c r="AG2" s="148"/>
       <c r="AH2" s="148"/>
     </row>
     <row r="3" spans="1:43" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="215" t="s">
+      <c r="B3" s="216" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="216"/>
+      <c r="C3" s="217"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="217" t="s">
+      <c r="E3" s="218" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="218"/>
-      <c r="G3" s="218"/>
-      <c r="H3" s="218"/>
-      <c r="I3" s="218"/>
-      <c r="J3" s="218"/>
+      <c r="F3" s="219"/>
+      <c r="G3" s="219"/>
+      <c r="H3" s="219"/>
+      <c r="I3" s="219"/>
+      <c r="J3" s="219"/>
       <c r="K3" s="74" t="s">
         <v>7</v>
       </c>
       <c r="L3" s="12"/>
-      <c r="M3" s="202" t="s">
+      <c r="M3" s="203" t="s">
         <v>4</v>
       </c>
-      <c r="N3" s="202"/>
+      <c r="N3" s="203"/>
       <c r="O3" s="141" t="s">
         <v>5</v>
       </c>
-      <c r="P3" s="202" t="s">
+      <c r="P3" s="203" t="s">
         <v>6</v>
       </c>
-      <c r="Q3" s="202"/>
-      <c r="R3" s="202"/>
-      <c r="S3" s="202"/>
-      <c r="T3" s="202"/>
-      <c r="U3" s="202"/>
-      <c r="V3" s="202"/>
-      <c r="W3" s="202"/>
-      <c r="X3" s="202"/>
-      <c r="Y3" s="202"/>
-      <c r="Z3" s="202" t="s">
+      <c r="Q3" s="203"/>
+      <c r="R3" s="203"/>
+      <c r="S3" s="203"/>
+      <c r="T3" s="203"/>
+      <c r="U3" s="203"/>
+      <c r="V3" s="203"/>
+      <c r="W3" s="203"/>
+      <c r="X3" s="203"/>
+      <c r="Y3" s="203"/>
+      <c r="Z3" s="203" t="s">
         <v>8</v>
       </c>
-      <c r="AA3" s="202"/>
-      <c r="AB3" s="202"/>
+      <c r="AA3" s="203"/>
+      <c r="AB3" s="203"/>
       <c r="AC3" s="141" t="s">
         <v>9</v>
       </c>
@@ -2885,7 +2903,7 @@
         <f>AA6-K6</f>
         <v>0</v>
       </c>
-      <c r="AC6" s="212"/>
+      <c r="AC6" s="213"/>
       <c r="AE6" s="20" t="s">
         <v>34</v>
       </c>
@@ -2986,7 +3004,7 @@
         <f t="shared" ref="AB7:AB10" si="5">AA7-K7</f>
         <v>0</v>
       </c>
-      <c r="AC7" s="212"/>
+      <c r="AC7" s="213"/>
       <c r="AF7" s="55"/>
       <c r="AG7" s="55"/>
       <c r="AH7" s="55"/>
@@ -3084,7 +3102,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC8" s="212"/>
+      <c r="AC8" s="213"/>
       <c r="AE8" s="152" t="s">
         <v>37</v>
       </c>
@@ -3194,7 +3212,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC9" s="212"/>
+      <c r="AC9" s="213"/>
       <c r="AE9" s="152" t="s">
         <v>43</v>
       </c>
@@ -3306,7 +3324,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC10" s="212"/>
+      <c r="AC10" s="213"/>
       <c r="AE10" s="152" t="s">
         <v>46</v>
       </c>
@@ -3426,7 +3444,7 @@
         <f t="shared" ref="AB11" si="13">Z11-K11</f>
         <v>0</v>
       </c>
-      <c r="AC11" s="213"/>
+      <c r="AC11" s="214"/>
       <c r="AD11" s="37"/>
       <c r="AE11" s="155" t="s">
         <v>49</v>
@@ -3467,8 +3485,8 @@
       <c r="J12" s="114"/>
       <c r="K12" s="68"/>
       <c r="L12" s="29"/>
-      <c r="M12" s="219"/>
-      <c r="N12" s="219"/>
+      <c r="M12" s="220"/>
+      <c r="N12" s="220"/>
       <c r="O12" s="113"/>
       <c r="P12" s="113"/>
       <c r="Q12" s="113"/>
@@ -3592,7 +3610,7 @@
         <f t="shared" ref="AB13:AB17" si="20">Z13-K13</f>
         <v>0</v>
       </c>
-      <c r="AC13" s="214"/>
+      <c r="AC13" s="215"/>
       <c r="AE13" s="167" t="s">
         <v>53</v>
       </c>
@@ -3701,7 +3719,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC14" s="212"/>
+      <c r="AC14" s="213"/>
       <c r="AE14" s="152" t="s">
         <v>23</v>
       </c>
@@ -3811,7 +3829,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC15" s="212"/>
+      <c r="AC15" s="213"/>
       <c r="AE15" s="171" t="s">
         <v>56</v>
       </c>
@@ -3922,7 +3940,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC16" s="212"/>
+      <c r="AC16" s="213"/>
       <c r="AE16" s="175" t="s">
         <v>57</v>
       </c>
@@ -4042,7 +4060,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC17" s="213"/>
+      <c r="AC17" s="214"/>
       <c r="AD17" s="37"/>
       <c r="AE17" s="152" t="s">
         <v>59</v>
@@ -4059,7 +4077,7 @@
         <f>AH16-AH15</f>
         <v>0</v>
       </c>
-      <c r="AI17" s="205" t="s">
+      <c r="AI17" s="206" t="s">
         <v>60</v>
       </c>
       <c r="AJ17" s="37"/>
@@ -4086,8 +4104,8 @@
       <c r="J18" s="120"/>
       <c r="K18" s="76"/>
       <c r="L18" s="51"/>
-      <c r="M18" s="204"/>
-      <c r="N18" s="204"/>
+      <c r="M18" s="205"/>
+      <c r="N18" s="205"/>
       <c r="O18" s="138"/>
       <c r="P18" s="119"/>
       <c r="Q18" s="119"/>
@@ -4103,13 +4121,13 @@
       <c r="AA18" s="76"/>
       <c r="AB18" s="76"/>
       <c r="AC18" s="44"/>
-      <c r="AE18" s="207" t="s">
+      <c r="AE18" s="208" t="s">
         <v>62</v>
       </c>
-      <c r="AF18" s="207"/>
-      <c r="AG18" s="207"/>
-      <c r="AH18" s="207"/>
-      <c r="AI18" s="206"/>
+      <c r="AF18" s="208"/>
+      <c r="AG18" s="208"/>
+      <c r="AH18" s="208"/>
+      <c r="AI18" s="207"/>
     </row>
     <row r="19" spans="1:43" s="19" customFormat="1" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A19" s="187" t="s">
@@ -4203,11 +4221,11 @@
         <v>0</v>
       </c>
       <c r="AC19" s="6"/>
-      <c r="AE19" s="208"/>
-      <c r="AF19" s="208"/>
-      <c r="AG19" s="208"/>
-      <c r="AH19" s="208"/>
-      <c r="AI19" s="206"/>
+      <c r="AE19" s="209"/>
+      <c r="AF19" s="209"/>
+      <c r="AG19" s="209"/>
+      <c r="AH19" s="209"/>
+      <c r="AI19" s="207"/>
     </row>
     <row r="20" spans="1:43" s="20" customFormat="1" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
@@ -4294,7 +4312,7 @@
       <c r="AF20" s="55"/>
       <c r="AG20" s="55"/>
       <c r="AH20" s="55"/>
-      <c r="AI20" s="206"/>
+      <c r="AI20" s="207"/>
     </row>
     <row r="21" spans="1:43" s="19" customFormat="1" ht="15.75" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A21" s="187" t="s">
@@ -5802,8 +5820,8 @@
       <c r="J38" s="126"/>
       <c r="K38" s="77"/>
       <c r="L38" s="51"/>
-      <c r="M38" s="201"/>
-      <c r="N38" s="201"/>
+      <c r="M38" s="202"/>
+      <c r="N38" s="202"/>
       <c r="O38" s="140"/>
       <c r="P38" s="125"/>
       <c r="Q38" s="125"/>
@@ -18365,22 +18383,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="220" t="s">
+      <c r="A1" s="201" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="220"/>
-      <c r="C1" s="220"/>
-      <c r="D1" s="220"/>
-      <c r="E1" s="220"/>
+      <c r="B1" s="201"/>
+      <c r="C1" s="201"/>
+      <c r="D1" s="201"/>
+      <c r="E1" s="201"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="220" t="s">
+      <c r="A2" s="201" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="220"/>
-      <c r="C2" s="220"/>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
+      <c r="B2" s="201"/>
+      <c r="C2" s="201"/>
+      <c r="D2" s="201"/>
+      <c r="E2" s="201"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
@@ -18461,11 +18479,53 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D7" s="200">
+        <v>46212</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>103</v>
+      </c>
+      <c r="G7" t="s">
+        <v>145</v>
+      </c>
       <c r="I7" s="180" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C8" t="s">
+        <v>147</v>
+      </c>
+      <c r="D8" s="200">
+        <v>46214</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G8" t="s">
+        <v>148</v>
+      </c>
       <c r="I8" s="181" t="s">
         <v>103</v>
       </c>
@@ -18510,26 +18570,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="220" t="s">
+      <c r="A1" s="201" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="220"/>
-      <c r="C1" s="220"/>
-      <c r="D1" s="220"/>
-      <c r="E1" s="220"/>
-      <c r="F1" s="220"/>
-      <c r="G1" s="220"/>
+      <c r="B1" s="201"/>
+      <c r="C1" s="201"/>
+      <c r="D1" s="201"/>
+      <c r="E1" s="201"/>
+      <c r="F1" s="201"/>
+      <c r="G1" s="201"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="220" t="s">
+      <c r="A2" s="201" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="220"/>
-      <c r="C2" s="220"/>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
-      <c r="F2" s="220"/>
-      <c r="G2" s="220"/>
+      <c r="B2" s="201"/>
+      <c r="C2" s="201"/>
+      <c r="D2" s="201"/>
+      <c r="E2" s="201"/>
+      <c r="F2" s="201"/>
+      <c r="G2" s="201"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
@@ -18630,7 +18690,7 @@
         <v>14</v>
       </c>
       <c r="H6" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="I6" s="19" t="s">
         <v>129</v>

</xml_diff>

<commit_message>
MAJ liste activites Sprint 2 - toutes les issues
</commit_message>
<xml_diff>
--- a/docs/TP2-FoxTrot-Liste_Activites-Sprint2.xlsx
+++ b/docs/TP2-FoxTrot-Liste_Activites-Sprint2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UQAM\Été 2026\INF6150 (Génie logiciel - Conduite de projets informatiques)\Travaux Pratiques\TP2\fixmycar\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29221729-89D3-48F5-BB5A-E3BCDFE2995D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACC31011-D03B-4E14-98F0-D0B2075E9E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Activités" sheetId="1" r:id="rId1"/>
@@ -1802,61 +1802,61 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="17" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="16" fontId="16" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="16" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="19" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="1" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="1" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="17" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1868,7 +1868,39 @@
     <cellStyle name="Normal 2" xfId="4" xr:uid="{952DC8A1-D8FF-4F17-A248-DB6C365AA9A7}"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{258B3E6A-1317-4862-A210-0F9DAE6EB1D0}"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="27">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2271,35 +2303,35 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3A12FB0F-C40A-B748-8030-98D340CFAB34}" name="Tableau2" displayName="Tableau2" ref="A4:G10" totalsRowShown="0" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3A12FB0F-C40A-B748-8030-98D340CFAB34}" name="Tableau2" displayName="Tableau2" ref="A4:G10" totalsRowShown="0" dataDxfId="15">
   <autoFilter ref="A4:G10" xr:uid="{8AE4CE81-0313-2046-8C9D-FC8A5BDAF35E}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{36580D9E-E44F-E144-9187-9D6816E7AD65}" name="No." dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{EF559DC7-F47B-9848-8130-B462D7345CF6}" name="Titre court" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{82194528-C6CF-814C-9068-B4CEE7AB8C8E}" name="Description" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{FD6B68BF-B7A7-6B4C-89C4-B008807F3FC2}" name="Date de création" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{9BF3BF16-17B1-F146-97D3-9D22567C832F}" name="Affecté à (initiales)" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{7AF9C5EC-5B6E-5C43-B14B-1BBD1D028344}" name="Statut" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{A53E42DA-438D-C749-AC68-3D736120C878}" name="Solution envisagée ou appliquée" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{36580D9E-E44F-E144-9187-9D6816E7AD65}" name="No." dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{EF559DC7-F47B-9848-8130-B462D7345CF6}" name="Titre court" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{82194528-C6CF-814C-9068-B4CEE7AB8C8E}" name="Description" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{FD6B68BF-B7A7-6B4C-89C4-B008807F3FC2}" name="Date de création" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{9BF3BF16-17B1-F146-97D3-9D22567C832F}" name="Affecté à (initiales)" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{7AF9C5EC-5B6E-5C43-B14B-1BBD1D028344}" name="Statut" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{A53E42DA-438D-C749-AC68-3D736120C878}" name="Solution envisagée ou appliquée" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B8EC000B-D60C-D54E-89A3-4DAFB6D317CF}" name="Tableau3" displayName="Tableau3" ref="A4:J9" totalsRowShown="0" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B8EC000B-D60C-D54E-89A3-4DAFB6D317CF}" name="Tableau3" displayName="Tableau3" ref="A4:J9" totalsRowShown="0" dataDxfId="26">
   <autoFilter ref="A4:J9" xr:uid="{E1E6DC87-7A9F-264E-BA03-CD93728E459B}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{700F170B-9E35-454D-B601-2C8F61AC472A}" name="No." dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{69AD1862-3369-2F48-9B47-23217AD6E1A7}" name="Titre court" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{1204722B-3D6B-0843-9A2E-7ED16DAED71A}" name="Description du risque" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{6CE70BC6-06C1-D24D-98D7-4A3E45D6488D}" name="Probabilité d'occurrence" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{C1803549-A0D1-3B45-A312-78E45EC1161F}" name="Niveau d'impact" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{AB57BB6B-52E7-7147-B89C-61E7504410DB}" name="Date de création" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{4A075D44-5451-5A41-8EB6-CFDC70386649}" name="Affecté à (initiales)" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{32D938AC-3C43-104A-96A5-6759770A9983}" name="Statut" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{9C3D641B-166E-7A4F-8FEA-A4067A23B751}" name="Plan(s) de mitigation" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{43F9D95D-A1C9-D540-AD50-99C65F9EF0BB}" name="Plan(s) de contingence" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{700F170B-9E35-454D-B601-2C8F61AC472A}" name="No." dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{69AD1862-3369-2F48-9B47-23217AD6E1A7}" name="Titre court" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{1204722B-3D6B-0843-9A2E-7ED16DAED71A}" name="Description du risque" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{6CE70BC6-06C1-D24D-98D7-4A3E45D6488D}" name="Probabilité d'occurrence" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{C1803549-A0D1-3B45-A312-78E45EC1161F}" name="Niveau d'impact" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{AB57BB6B-52E7-7147-B89C-61E7504410DB}" name="Date de création" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{4A075D44-5451-5A41-8EB6-CFDC70386649}" name="Affecté à (initiales)" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{32D938AC-3C43-104A-96A5-6759770A9983}" name="Statut" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{9C3D641B-166E-7A4F-8FEA-A4067A23B751}" name="Plan(s) de mitigation" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{43F9D95D-A1C9-D540-AD50-99C65F9EF0BB}" name="Plan(s) de contingence" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2556,120 +2588,120 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="210" t="s">
+      <c r="B1" s="206" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="210"/>
-      <c r="D1" s="210"/>
-      <c r="E1" s="210"/>
-      <c r="F1" s="210"/>
-      <c r="G1" s="210"/>
-      <c r="H1" s="210"/>
-      <c r="I1" s="210"/>
-      <c r="J1" s="210"/>
-      <c r="K1" s="210"/>
+      <c r="C1" s="206"/>
+      <c r="D1" s="206"/>
+      <c r="E1" s="206"/>
+      <c r="F1" s="206"/>
+      <c r="G1" s="206"/>
+      <c r="H1" s="206"/>
+      <c r="I1" s="206"/>
+      <c r="J1" s="206"/>
+      <c r="K1" s="206"/>
       <c r="L1" s="11"/>
-      <c r="M1" s="212" t="s">
+      <c r="M1" s="208" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="212"/>
-      <c r="O1" s="212"/>
-      <c r="P1" s="212"/>
-      <c r="Q1" s="212"/>
-      <c r="R1" s="212"/>
-      <c r="S1" s="212"/>
-      <c r="T1" s="212"/>
-      <c r="U1" s="212"/>
-      <c r="V1" s="212"/>
-      <c r="W1" s="212"/>
-      <c r="X1" s="212"/>
-      <c r="Y1" s="212"/>
-      <c r="Z1" s="212"/>
-      <c r="AA1" s="212"/>
-      <c r="AB1" s="212"/>
-      <c r="AC1" s="212"/>
+      <c r="N1" s="208"/>
+      <c r="O1" s="208"/>
+      <c r="P1" s="208"/>
+      <c r="Q1" s="208"/>
+      <c r="R1" s="208"/>
+      <c r="S1" s="208"/>
+      <c r="T1" s="208"/>
+      <c r="U1" s="208"/>
+      <c r="V1" s="208"/>
+      <c r="W1" s="208"/>
+      <c r="X1" s="208"/>
+      <c r="Y1" s="208"/>
+      <c r="Z1" s="208"/>
+      <c r="AA1" s="208"/>
+      <c r="AB1" s="208"/>
+      <c r="AC1" s="208"/>
     </row>
     <row r="2" spans="1:43" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="204" t="s">
+      <c r="B2" s="219" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="204"/>
-      <c r="D2" s="204"/>
-      <c r="E2" s="204"/>
-      <c r="F2" s="204"/>
-      <c r="G2" s="204"/>
-      <c r="H2" s="204"/>
-      <c r="I2" s="204"/>
-      <c r="J2" s="204"/>
-      <c r="K2" s="204"/>
+      <c r="C2" s="219"/>
+      <c r="D2" s="219"/>
+      <c r="E2" s="219"/>
+      <c r="F2" s="219"/>
+      <c r="G2" s="219"/>
+      <c r="H2" s="219"/>
+      <c r="I2" s="219"/>
+      <c r="J2" s="219"/>
+      <c r="K2" s="219"/>
       <c r="L2" s="54"/>
-      <c r="M2" s="211" t="s">
+      <c r="M2" s="207" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="211"/>
-      <c r="O2" s="211"/>
-      <c r="P2" s="211"/>
-      <c r="Q2" s="211"/>
-      <c r="R2" s="211"/>
-      <c r="S2" s="211"/>
-      <c r="T2" s="211"/>
-      <c r="U2" s="211"/>
-      <c r="V2" s="211"/>
-      <c r="W2" s="211"/>
-      <c r="X2" s="211"/>
-      <c r="Y2" s="211"/>
-      <c r="Z2" s="211"/>
-      <c r="AA2" s="211"/>
-      <c r="AB2" s="211"/>
-      <c r="AC2" s="211"/>
+      <c r="N2" s="207"/>
+      <c r="O2" s="207"/>
+      <c r="P2" s="207"/>
+      <c r="Q2" s="207"/>
+      <c r="R2" s="207"/>
+      <c r="S2" s="207"/>
+      <c r="T2" s="207"/>
+      <c r="U2" s="207"/>
+      <c r="V2" s="207"/>
+      <c r="W2" s="207"/>
+      <c r="X2" s="207"/>
+      <c r="Y2" s="207"/>
+      <c r="Z2" s="207"/>
+      <c r="AA2" s="207"/>
+      <c r="AB2" s="207"/>
+      <c r="AC2" s="207"/>
       <c r="AF2" s="148"/>
       <c r="AG2" s="148"/>
       <c r="AH2" s="148"/>
     </row>
     <row r="3" spans="1:43" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="216" t="s">
+      <c r="B3" s="212" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="217"/>
+      <c r="C3" s="213"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="218" t="s">
+      <c r="E3" s="214" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="219"/>
-      <c r="G3" s="219"/>
-      <c r="H3" s="219"/>
-      <c r="I3" s="219"/>
-      <c r="J3" s="219"/>
+      <c r="F3" s="215"/>
+      <c r="G3" s="215"/>
+      <c r="H3" s="215"/>
+      <c r="I3" s="215"/>
+      <c r="J3" s="215"/>
       <c r="K3" s="74" t="s">
         <v>7</v>
       </c>
       <c r="L3" s="12"/>
-      <c r="M3" s="203" t="s">
+      <c r="M3" s="216" t="s">
         <v>4</v>
       </c>
-      <c r="N3" s="203"/>
+      <c r="N3" s="216"/>
       <c r="O3" s="141" t="s">
         <v>5</v>
       </c>
-      <c r="P3" s="203" t="s">
+      <c r="P3" s="216" t="s">
         <v>6</v>
       </c>
-      <c r="Q3" s="203"/>
-      <c r="R3" s="203"/>
-      <c r="S3" s="203"/>
-      <c r="T3" s="203"/>
-      <c r="U3" s="203"/>
-      <c r="V3" s="203"/>
-      <c r="W3" s="203"/>
-      <c r="X3" s="203"/>
-      <c r="Y3" s="203"/>
-      <c r="Z3" s="203" t="s">
+      <c r="Q3" s="216"/>
+      <c r="R3" s="216"/>
+      <c r="S3" s="216"/>
+      <c r="T3" s="216"/>
+      <c r="U3" s="216"/>
+      <c r="V3" s="216"/>
+      <c r="W3" s="216"/>
+      <c r="X3" s="216"/>
+      <c r="Y3" s="216"/>
+      <c r="Z3" s="216" t="s">
         <v>8</v>
       </c>
-      <c r="AA3" s="203"/>
-      <c r="AB3" s="203"/>
+      <c r="AA3" s="216"/>
+      <c r="AB3" s="216"/>
       <c r="AC3" s="141" t="s">
         <v>9</v>
       </c>
@@ -2903,7 +2935,7 @@
         <f>AA6-K6</f>
         <v>0</v>
       </c>
-      <c r="AC6" s="213"/>
+      <c r="AC6" s="209"/>
       <c r="AE6" s="20" t="s">
         <v>34</v>
       </c>
@@ -3004,7 +3036,7 @@
         <f t="shared" ref="AB7:AB10" si="5">AA7-K7</f>
         <v>0</v>
       </c>
-      <c r="AC7" s="213"/>
+      <c r="AC7" s="209"/>
       <c r="AF7" s="55"/>
       <c r="AG7" s="55"/>
       <c r="AH7" s="55"/>
@@ -3102,7 +3134,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC8" s="213"/>
+      <c r="AC8" s="209"/>
       <c r="AE8" s="152" t="s">
         <v>37</v>
       </c>
@@ -3212,7 +3244,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC9" s="213"/>
+      <c r="AC9" s="209"/>
       <c r="AE9" s="152" t="s">
         <v>43</v>
       </c>
@@ -3324,7 +3356,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC10" s="213"/>
+      <c r="AC10" s="209"/>
       <c r="AE10" s="152" t="s">
         <v>46</v>
       </c>
@@ -3444,18 +3476,18 @@
         <f t="shared" ref="AB11" si="13">Z11-K11</f>
         <v>0</v>
       </c>
-      <c r="AC11" s="214"/>
+      <c r="AC11" s="210"/>
       <c r="AD11" s="37"/>
       <c r="AE11" s="155" t="s">
         <v>49</v>
       </c>
       <c r="AF11" s="156">
         <f>U37</f>
-        <v>26</v>
+        <v>119</v>
       </c>
       <c r="AG11" s="162">
         <f>Z37</f>
-        <v>2860</v>
+        <v>13090</v>
       </c>
       <c r="AH11" s="157">
         <v>9</v>
@@ -3485,8 +3517,8 @@
       <c r="J12" s="114"/>
       <c r="K12" s="68"/>
       <c r="L12" s="29"/>
-      <c r="M12" s="220"/>
-      <c r="N12" s="220"/>
+      <c r="M12" s="217"/>
+      <c r="N12" s="217"/>
       <c r="O12" s="113"/>
       <c r="P12" s="113"/>
       <c r="Q12" s="113"/>
@@ -3610,17 +3642,17 @@
         <f t="shared" ref="AB13:AB17" si="20">Z13-K13</f>
         <v>0</v>
       </c>
-      <c r="AC13" s="215"/>
+      <c r="AC13" s="211"/>
       <c r="AE13" s="167" t="s">
         <v>53</v>
       </c>
       <c r="AF13" s="168">
         <f>U45</f>
-        <v>94</v>
+        <v>187</v>
       </c>
       <c r="AG13" s="169">
         <f>Z45</f>
-        <v>10340</v>
+        <v>20570</v>
       </c>
       <c r="AH13" s="170">
         <v>2</v>
@@ -3719,17 +3751,17 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC14" s="213"/>
+      <c r="AC14" s="209"/>
       <c r="AE14" s="152" t="s">
         <v>23</v>
       </c>
       <c r="AF14" s="154">
         <f>V45</f>
-        <v>244</v>
+        <v>151</v>
       </c>
       <c r="AG14" s="161">
         <f>V45*tarif</f>
-        <v>26840</v>
+        <v>16610</v>
       </c>
       <c r="AH14" s="153">
         <v>7</v>
@@ -3829,7 +3861,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC15" s="213"/>
+      <c r="AC15" s="209"/>
       <c r="AE15" s="171" t="s">
         <v>56</v>
       </c>
@@ -3940,7 +3972,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC16" s="213"/>
+      <c r="AC16" s="209"/>
       <c r="AE16" s="175" t="s">
         <v>57</v>
       </c>
@@ -4060,7 +4092,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC17" s="214"/>
+      <c r="AC17" s="210"/>
       <c r="AD17" s="37"/>
       <c r="AE17" s="152" t="s">
         <v>59</v>
@@ -4077,7 +4109,7 @@
         <f>AH16-AH15</f>
         <v>0</v>
       </c>
-      <c r="AI17" s="206" t="s">
+      <c r="AI17" s="202" t="s">
         <v>60</v>
       </c>
       <c r="AJ17" s="37"/>
@@ -4104,8 +4136,8 @@
       <c r="J18" s="120"/>
       <c r="K18" s="76"/>
       <c r="L18" s="51"/>
-      <c r="M18" s="205"/>
-      <c r="N18" s="205"/>
+      <c r="M18" s="220"/>
+      <c r="N18" s="220"/>
       <c r="O18" s="138"/>
       <c r="P18" s="119"/>
       <c r="Q18" s="119"/>
@@ -4121,13 +4153,13 @@
       <c r="AA18" s="76"/>
       <c r="AB18" s="76"/>
       <c r="AC18" s="44"/>
-      <c r="AE18" s="208" t="s">
+      <c r="AE18" s="204" t="s">
         <v>62</v>
       </c>
-      <c r="AF18" s="208"/>
-      <c r="AG18" s="208"/>
-      <c r="AH18" s="208"/>
-      <c r="AI18" s="207"/>
+      <c r="AF18" s="204"/>
+      <c r="AG18" s="204"/>
+      <c r="AH18" s="204"/>
+      <c r="AI18" s="203"/>
     </row>
     <row r="19" spans="1:43" s="19" customFormat="1" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A19" s="187" t="s">
@@ -4170,7 +4202,7 @@
         <v>46212</v>
       </c>
       <c r="N19" s="136">
-        <f t="shared" ref="N19:N36" si="27">M19-C19</f>
+        <f t="shared" ref="N19:N22" si="27">M19-C19</f>
         <v>18</v>
       </c>
       <c r="O19" s="121"/>
@@ -4190,7 +4222,7 @@
         <v>2</v>
       </c>
       <c r="U19" s="137">
-        <f t="shared" ref="U19:U36" si="28">SUM(P19:T19)</f>
+        <f t="shared" ref="U19:U22" si="28">SUM(P19:T19)</f>
         <v>13</v>
       </c>
       <c r="V19" s="131">
@@ -4198,11 +4230,11 @@
         <v>0</v>
       </c>
       <c r="W19" s="137">
-        <f t="shared" ref="W19:W36" si="29">U19+V19</f>
+        <f t="shared" ref="W19:W22" si="29">U19+V19</f>
         <v>13</v>
       </c>
       <c r="X19" s="131" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="Y19" s="137">
         <f t="shared" ref="Y19:Y36" si="30">(W19-J19)</f>
@@ -4221,11 +4253,11 @@
         <v>0</v>
       </c>
       <c r="AC19" s="6"/>
-      <c r="AE19" s="209"/>
-      <c r="AF19" s="209"/>
-      <c r="AG19" s="209"/>
-      <c r="AH19" s="209"/>
-      <c r="AI19" s="207"/>
+      <c r="AE19" s="205"/>
+      <c r="AF19" s="205"/>
+      <c r="AG19" s="205"/>
+      <c r="AH19" s="205"/>
+      <c r="AI19" s="203"/>
     </row>
     <row r="20" spans="1:43" s="20" customFormat="1" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
@@ -4264,31 +4296,43 @@
         <v>1320</v>
       </c>
       <c r="L20" s="9"/>
-      <c r="M20" s="106"/>
+      <c r="M20" s="106">
+        <v>46210</v>
+      </c>
       <c r="N20" s="136">
         <f t="shared" si="27"/>
-        <v>-46194</v>
+        <v>16</v>
       </c>
       <c r="O20" s="142"/>
-      <c r="P20" s="131"/>
-      <c r="Q20" s="131"/>
-      <c r="R20" s="131"/>
-      <c r="S20" s="131"/>
-      <c r="T20" s="131"/>
+      <c r="P20" s="131">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="131">
+        <v>1</v>
+      </c>
+      <c r="R20" s="131">
+        <v>1</v>
+      </c>
+      <c r="S20" s="131">
+        <v>1</v>
+      </c>
+      <c r="T20" s="131">
+        <v>8</v>
+      </c>
       <c r="U20" s="137">
         <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="V20" s="131">
+        <f t="shared" ref="V20:V22" si="34">J20-U20</f>
         <v>0</v>
-      </c>
-      <c r="V20" s="131">
-        <f t="shared" ref="V20:V36" si="34">J20-U20</f>
-        <v>12</v>
       </c>
       <c r="W20" s="137">
         <f t="shared" si="29"/>
         <v>12</v>
       </c>
       <c r="X20" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y20" s="137">
         <f t="shared" si="30"/>
@@ -4296,7 +4340,7 @@
       </c>
       <c r="Z20" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1320</v>
       </c>
       <c r="AA20" s="109">
         <f t="shared" si="32"/>
@@ -4304,7 +4348,7 @@
       </c>
       <c r="AB20" s="139">
         <f t="shared" ref="AB20:AB36" si="35">Z20-K20</f>
-        <v>-1320</v>
+        <v>0</v>
       </c>
       <c r="AC20" s="6"/>
       <c r="AD20" s="19"/>
@@ -4312,7 +4356,7 @@
       <c r="AF20" s="55"/>
       <c r="AG20" s="55"/>
       <c r="AH20" s="55"/>
-      <c r="AI20" s="207"/>
+      <c r="AI20" s="203"/>
     </row>
     <row r="21" spans="1:43" s="19" customFormat="1" ht="15.75" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A21" s="187" t="s">
@@ -4351,31 +4395,43 @@
         <v>1540</v>
       </c>
       <c r="L21" s="9"/>
-      <c r="M21" s="106"/>
+      <c r="M21" s="106">
+        <v>46210</v>
+      </c>
       <c r="N21" s="136">
         <f t="shared" si="27"/>
-        <v>-46194</v>
+        <v>16</v>
       </c>
       <c r="O21" s="142"/>
-      <c r="P21" s="131"/>
-      <c r="Q21" s="131"/>
-      <c r="R21" s="131"/>
-      <c r="S21" s="131"/>
-      <c r="T21" s="131"/>
+      <c r="P21" s="131">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="131">
+        <v>2</v>
+      </c>
+      <c r="R21" s="131">
+        <v>1</v>
+      </c>
+      <c r="S21" s="131">
+        <v>9</v>
+      </c>
+      <c r="T21" s="131">
+        <v>1</v>
+      </c>
       <c r="U21" s="137">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="V21" s="131">
         <f t="shared" si="34"/>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="W21" s="137">
         <f t="shared" si="29"/>
         <v>14</v>
       </c>
       <c r="X21" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y21" s="137">
         <f t="shared" si="30"/>
@@ -4383,7 +4439,7 @@
       </c>
       <c r="Z21" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1540</v>
       </c>
       <c r="AA21" s="109">
         <f t="shared" si="32"/>
@@ -4391,7 +4447,7 @@
       </c>
       <c r="AB21" s="139">
         <f t="shared" si="35"/>
-        <v>-1540</v>
+        <v>0</v>
       </c>
       <c r="AC21" s="6"/>
       <c r="AF21" s="55"/>
@@ -4436,31 +4492,43 @@
         <v>1430</v>
       </c>
       <c r="L22" s="9"/>
-      <c r="M22" s="106"/>
+      <c r="M22" s="106">
+        <v>46209</v>
+      </c>
       <c r="N22" s="136">
         <f t="shared" si="27"/>
-        <v>-46194</v>
+        <v>15</v>
       </c>
       <c r="O22" s="142"/>
-      <c r="P22" s="131"/>
-      <c r="Q22" s="131"/>
-      <c r="R22" s="131"/>
-      <c r="S22" s="131"/>
-      <c r="T22" s="131"/>
+      <c r="P22" s="131">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="131">
+        <v>9</v>
+      </c>
+      <c r="R22" s="131">
+        <v>1</v>
+      </c>
+      <c r="S22" s="131">
+        <v>1</v>
+      </c>
+      <c r="T22" s="131">
+        <v>1</v>
+      </c>
       <c r="U22" s="137">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="V22" s="131">
         <f t="shared" si="34"/>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="W22" s="137">
         <f t="shared" si="29"/>
         <v>13</v>
       </c>
       <c r="X22" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y22" s="137">
         <f t="shared" si="30"/>
@@ -4468,7 +4536,7 @@
       </c>
       <c r="Z22" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1430</v>
       </c>
       <c r="AA22" s="109">
         <f t="shared" si="32"/>
@@ -4476,7 +4544,7 @@
       </c>
       <c r="AB22" s="139">
         <f t="shared" si="35"/>
-        <v>-1430</v>
+        <v>0</v>
       </c>
       <c r="AC22" s="6"/>
       <c r="AF22" s="55"/>
@@ -4520,31 +4588,43 @@
         <v>1430</v>
       </c>
       <c r="L23" s="9"/>
-      <c r="M23" s="106"/>
+      <c r="M23" s="106">
+        <v>46212</v>
+      </c>
       <c r="N23" s="136">
-        <f t="shared" si="27"/>
-        <v>-46215</v>
+        <f t="shared" ref="N19:N36" si="36">M23-C23</f>
+        <v>-3</v>
       </c>
       <c r="O23" s="142"/>
-      <c r="P23" s="131"/>
-      <c r="Q23" s="131"/>
-      <c r="R23" s="131"/>
-      <c r="S23" s="131"/>
-      <c r="T23" s="131"/>
+      <c r="P23" s="131">
+        <v>2</v>
+      </c>
+      <c r="Q23" s="131">
+        <v>1</v>
+      </c>
+      <c r="R23" s="131">
+        <v>1</v>
+      </c>
+      <c r="S23" s="131">
+        <v>7</v>
+      </c>
+      <c r="T23" s="131">
+        <v>2</v>
+      </c>
       <c r="U23" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" ref="U19:U36" si="37">SUM(P23:T23)</f>
+        <v>13</v>
+      </c>
+      <c r="V23" s="131">
+        <f t="shared" ref="V20:V36" si="38">J23-U23</f>
         <v>0</v>
       </c>
-      <c r="V23" s="131">
-        <f t="shared" si="34"/>
+      <c r="W23" s="137">
+        <f t="shared" ref="W19:W36" si="39">U23+V23</f>
         <v>13</v>
       </c>
-      <c r="W23" s="137">
-        <f t="shared" si="29"/>
-        <v>13</v>
-      </c>
       <c r="X23" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y23" s="137">
         <f t="shared" si="30"/>
@@ -4552,7 +4632,7 @@
       </c>
       <c r="Z23" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1430</v>
       </c>
       <c r="AA23" s="109">
         <f t="shared" si="32"/>
@@ -4560,7 +4640,7 @@
       </c>
       <c r="AB23" s="139">
         <f t="shared" si="35"/>
-        <v>-1430</v>
+        <v>0</v>
       </c>
       <c r="AC23" s="6"/>
       <c r="AF23" s="55"/>
@@ -4604,31 +4684,43 @@
         <v>1540</v>
       </c>
       <c r="L24" s="9"/>
-      <c r="M24" s="106"/>
+      <c r="M24" s="106">
+        <v>46213</v>
+      </c>
       <c r="N24" s="136">
-        <f t="shared" si="27"/>
-        <v>-46215</v>
+        <f t="shared" si="36"/>
+        <v>-2</v>
       </c>
       <c r="O24" s="121"/>
-      <c r="P24" s="131"/>
-      <c r="Q24" s="131"/>
-      <c r="R24" s="131"/>
-      <c r="S24" s="131"/>
-      <c r="T24" s="131"/>
+      <c r="P24" s="131">
+        <v>1.5</v>
+      </c>
+      <c r="Q24" s="131">
+        <v>1</v>
+      </c>
+      <c r="R24" s="131">
+        <v>9.5</v>
+      </c>
+      <c r="S24" s="131">
+        <v>1</v>
+      </c>
+      <c r="T24" s="131">
+        <v>1</v>
+      </c>
       <c r="U24" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
+        <v>14</v>
+      </c>
+      <c r="V24" s="131">
+        <f t="shared" si="38"/>
         <v>0</v>
       </c>
-      <c r="V24" s="131">
-        <f t="shared" si="34"/>
+      <c r="W24" s="137">
+        <f t="shared" si="39"/>
         <v>14</v>
       </c>
-      <c r="W24" s="137">
-        <f t="shared" si="29"/>
-        <v>14</v>
-      </c>
       <c r="X24" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y24" s="137">
         <f t="shared" si="30"/>
@@ -4636,7 +4728,7 @@
       </c>
       <c r="Z24" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1540</v>
       </c>
       <c r="AA24" s="109">
         <f t="shared" si="32"/>
@@ -4644,7 +4736,7 @@
       </c>
       <c r="AB24" s="139">
         <f t="shared" si="35"/>
-        <v>-1540</v>
+        <v>0</v>
       </c>
       <c r="AC24" s="6"/>
       <c r="AD24" s="19"/>
@@ -4691,31 +4783,43 @@
         <v>1540</v>
       </c>
       <c r="L25" s="9"/>
-      <c r="M25" s="106"/>
+      <c r="M25" s="106">
+        <v>46215</v>
+      </c>
       <c r="N25" s="136">
-        <f t="shared" si="27"/>
-        <v>-46215</v>
+        <f t="shared" si="36"/>
+        <v>0</v>
       </c>
       <c r="O25" s="121"/>
-      <c r="P25" s="131"/>
-      <c r="Q25" s="131"/>
-      <c r="R25" s="131"/>
-      <c r="S25" s="131"/>
-      <c r="T25" s="131"/>
+      <c r="P25" s="131">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="131">
+        <v>2</v>
+      </c>
+      <c r="R25" s="131">
+        <v>8.5</v>
+      </c>
+      <c r="S25" s="131">
+        <v>1</v>
+      </c>
+      <c r="T25" s="131">
+        <v>1.5</v>
+      </c>
       <c r="U25" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
+        <v>14</v>
+      </c>
+      <c r="V25" s="131">
+        <f t="shared" si="38"/>
         <v>0</v>
       </c>
-      <c r="V25" s="131">
-        <f t="shared" si="34"/>
+      <c r="W25" s="137">
+        <f t="shared" si="39"/>
         <v>14</v>
       </c>
-      <c r="W25" s="137">
-        <f t="shared" si="29"/>
-        <v>14</v>
-      </c>
       <c r="X25" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y25" s="137">
         <f t="shared" si="30"/>
@@ -4723,7 +4827,7 @@
       </c>
       <c r="Z25" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1540</v>
       </c>
       <c r="AA25" s="109">
         <f t="shared" si="32"/>
@@ -4731,7 +4835,7 @@
       </c>
       <c r="AB25" s="139">
         <f t="shared" si="35"/>
-        <v>-1540</v>
+        <v>0</v>
       </c>
       <c r="AC25" s="6"/>
       <c r="AF25" s="55"/>
@@ -4780,7 +4884,7 @@
         <v>46213</v>
       </c>
       <c r="N26" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-2</v>
       </c>
       <c r="O26" s="121"/>
@@ -4788,27 +4892,27 @@
         <v>7</v>
       </c>
       <c r="Q26" s="131">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R26" s="131">
         <v>2</v>
       </c>
       <c r="S26" s="131">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T26" s="131">
         <v>1</v>
       </c>
       <c r="U26" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>13</v>
       </c>
       <c r="V26" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>0</v>
       </c>
       <c r="W26" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>13</v>
       </c>
       <c r="X26" s="131" t="s">
@@ -4872,31 +4976,43 @@
         <v>1210</v>
       </c>
       <c r="L27" s="9"/>
-      <c r="M27" s="106"/>
+      <c r="M27" s="106">
+        <v>46215</v>
+      </c>
       <c r="N27" s="136">
-        <f t="shared" si="27"/>
-        <v>-46215</v>
+        <f t="shared" si="36"/>
+        <v>0</v>
       </c>
       <c r="O27" s="121"/>
-      <c r="P27" s="131"/>
-      <c r="Q27" s="131"/>
-      <c r="R27" s="131"/>
-      <c r="S27" s="131"/>
-      <c r="T27" s="131"/>
+      <c r="P27" s="131">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="131">
+        <v>9</v>
+      </c>
+      <c r="R27" s="131">
+        <v>1</v>
+      </c>
+      <c r="S27" s="131">
+        <v>1</v>
+      </c>
+      <c r="T27" s="131">
+        <v>1</v>
+      </c>
       <c r="U27" s="137">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <f t="shared" si="37"/>
+        <v>13</v>
       </c>
       <c r="V27" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
+        <v>-2</v>
+      </c>
+      <c r="W27" s="137">
+        <f t="shared" si="39"/>
         <v>11</v>
       </c>
-      <c r="W27" s="137">
-        <f t="shared" si="29"/>
-        <v>11</v>
-      </c>
       <c r="X27" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y27" s="137">
         <f t="shared" si="30"/>
@@ -4904,7 +5020,7 @@
       </c>
       <c r="Z27" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1430</v>
       </c>
       <c r="AA27" s="109">
         <f t="shared" si="32"/>
@@ -4912,7 +5028,7 @@
       </c>
       <c r="AB27" s="139">
         <f t="shared" si="35"/>
-        <v>-1210</v>
+        <v>220</v>
       </c>
       <c r="AC27" s="6"/>
       <c r="AF27" s="55"/>
@@ -4958,7 +5074,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="106"/>
       <c r="N28" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-46215</v>
       </c>
       <c r="O28" s="121"/>
@@ -4968,19 +5084,19 @@
       <c r="S28" s="131"/>
       <c r="T28" s="131"/>
       <c r="U28" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="V28" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>12</v>
       </c>
       <c r="W28" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>12</v>
       </c>
       <c r="X28" s="131" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="Y28" s="137">
         <f t="shared" si="30"/>
@@ -5045,7 +5161,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="106"/>
       <c r="N29" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-46236</v>
       </c>
       <c r="O29" s="121"/>
@@ -5055,15 +5171,15 @@
       <c r="S29" s="131"/>
       <c r="T29" s="131"/>
       <c r="U29" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="V29" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>10</v>
       </c>
       <c r="W29" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>10</v>
       </c>
       <c r="X29" s="131" t="s">
@@ -5130,7 +5246,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="106"/>
       <c r="N30" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-46236</v>
       </c>
       <c r="O30" s="121"/>
@@ -5140,15 +5256,15 @@
       <c r="S30" s="131"/>
       <c r="T30" s="131"/>
       <c r="U30" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="V30" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>15</v>
       </c>
       <c r="W30" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>15</v>
       </c>
       <c r="X30" s="131" t="s">
@@ -5214,7 +5330,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="106"/>
       <c r="N31" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-46236</v>
       </c>
       <c r="O31" s="121"/>
@@ -5224,15 +5340,15 @@
       <c r="S31" s="131"/>
       <c r="T31" s="131"/>
       <c r="U31" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="V31" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>12</v>
       </c>
       <c r="W31" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>12</v>
       </c>
       <c r="X31" s="131" t="s">
@@ -5298,7 +5414,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="106"/>
       <c r="N32" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-46236</v>
       </c>
       <c r="O32" s="121"/>
@@ -5308,15 +5424,15 @@
       <c r="S32" s="131"/>
       <c r="T32" s="131"/>
       <c r="U32" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="V32" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>12</v>
       </c>
       <c r="W32" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>12</v>
       </c>
       <c r="X32" s="131" t="s">
@@ -5385,7 +5501,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="106"/>
       <c r="N33" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-46236</v>
       </c>
       <c r="O33" s="121"/>
@@ -5395,15 +5511,15 @@
       <c r="S33" s="131"/>
       <c r="T33" s="131"/>
       <c r="U33" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="V33" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>15</v>
       </c>
       <c r="W33" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>15</v>
       </c>
       <c r="X33" s="131" t="s">
@@ -5470,7 +5586,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="106"/>
       <c r="N34" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-46236</v>
       </c>
       <c r="O34" s="121"/>
@@ -5480,15 +5596,15 @@
       <c r="S34" s="131"/>
       <c r="T34" s="131"/>
       <c r="U34" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="V34" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>12</v>
       </c>
       <c r="W34" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>12</v>
       </c>
       <c r="X34" s="131" t="s">
@@ -5554,7 +5670,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="106"/>
       <c r="N35" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-46236</v>
       </c>
       <c r="O35" s="121"/>
@@ -5564,15 +5680,15 @@
       <c r="S35" s="131"/>
       <c r="T35" s="131"/>
       <c r="U35" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="V35" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>11</v>
       </c>
       <c r="W35" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>11</v>
       </c>
       <c r="X35" s="131" t="s">
@@ -5638,7 +5754,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="106"/>
       <c r="N36" s="136">
-        <f t="shared" si="27"/>
+        <f t="shared" si="36"/>
         <v>-46236</v>
       </c>
       <c r="O36" s="121"/>
@@ -5648,15 +5764,15 @@
       <c r="S36" s="131"/>
       <c r="T36" s="131"/>
       <c r="U36" s="137">
-        <f t="shared" si="28"/>
+        <f t="shared" si="37"/>
         <v>0</v>
       </c>
       <c r="V36" s="131">
-        <f t="shared" si="34"/>
+        <f t="shared" si="38"/>
         <v>14</v>
       </c>
       <c r="W36" s="137">
-        <f t="shared" si="29"/>
+        <f t="shared" si="39"/>
         <v>14</v>
       </c>
       <c r="X36" s="131" t="s">
@@ -5700,27 +5816,27 @@
         <v>29</v>
       </c>
       <c r="E37" s="85">
-        <f t="shared" ref="E37:J37" si="36">SUM(E19:E36)</f>
+        <f t="shared" ref="E37:J37" si="40">SUM(E19:E36)</f>
         <v>46</v>
       </c>
       <c r="F37" s="85">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>41</v>
       </c>
       <c r="G37" s="85">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>40</v>
       </c>
       <c r="H37" s="85">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>45</v>
       </c>
       <c r="I37" s="85">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>58</v>
       </c>
       <c r="J37" s="85">
-        <f t="shared" si="36"/>
+        <f t="shared" si="40"/>
         <v>230</v>
       </c>
       <c r="K37" s="70">
@@ -5730,43 +5846,43 @@
       <c r="L37" s="49"/>
       <c r="M37" s="46">
         <f>MAX(M19:M36)</f>
-        <v>46213</v>
+        <v>46215</v>
       </c>
       <c r="N37" s="48">
         <f>M37-C37</f>
-        <v>-23</v>
+        <v>-21</v>
       </c>
       <c r="O37" s="47">
         <f>SUM(O21:O23)</f>
         <v>0</v>
       </c>
       <c r="P37" s="48">
-        <f t="shared" ref="P37:Y37" si="37">SUM(P19:P19)</f>
+        <f t="shared" ref="P37:Y37" si="41">SUM(P19:P19)</f>
         <v>8</v>
       </c>
       <c r="Q37" s="48">
-        <f t="shared" si="37"/>
+        <f t="shared" si="41"/>
         <v>1</v>
       </c>
       <c r="R37" s="48">
-        <f t="shared" si="37"/>
+        <f t="shared" si="41"/>
         <v>1</v>
       </c>
       <c r="S37" s="48">
-        <f t="shared" si="37"/>
+        <f t="shared" si="41"/>
         <v>1</v>
       </c>
       <c r="T37" s="48">
-        <f t="shared" si="37"/>
+        <f t="shared" si="41"/>
         <v>2</v>
       </c>
       <c r="U37" s="48">
         <f>SUM(U19:U36)</f>
-        <v>26</v>
+        <v>119</v>
       </c>
       <c r="V37" s="48">
         <f>SUM(V19:V36)</f>
-        <v>204</v>
+        <v>111</v>
       </c>
       <c r="W37" s="48">
         <f>SUM(W19:W36)</f>
@@ -5774,12 +5890,12 @@
       </c>
       <c r="X37" s="48"/>
       <c r="Y37" s="48">
-        <f t="shared" si="37"/>
+        <f t="shared" si="41"/>
         <v>0</v>
       </c>
       <c r="Z37" s="70">
-        <f t="shared" ref="Z37" si="38">tarif*U37</f>
-        <v>2860</v>
+        <f t="shared" ref="Z37" si="42">tarif*U37</f>
+        <v>13090</v>
       </c>
       <c r="AA37" s="70">
         <f t="shared" si="32"/>
@@ -5787,7 +5903,7 @@
       </c>
       <c r="AB37" s="70">
         <f t="shared" si="33"/>
-        <v>-22440</v>
+        <v>-12210</v>
       </c>
       <c r="AC37" s="50"/>
       <c r="AD37" s="37"/>
@@ -5820,8 +5936,8 @@
       <c r="J38" s="126"/>
       <c r="K38" s="77"/>
       <c r="L38" s="51"/>
-      <c r="M38" s="202"/>
-      <c r="N38" s="202"/>
+      <c r="M38" s="218"/>
+      <c r="N38" s="218"/>
       <c r="O38" s="140"/>
       <c r="P38" s="125"/>
       <c r="Q38" s="125"/>
@@ -5872,7 +5988,7 @@
         <v>1</v>
       </c>
       <c r="J39" s="108">
-        <f t="shared" ref="J39:J43" si="39">SUM(E39:I39)</f>
+        <f t="shared" ref="J39:J43" si="43">SUM(E39:I39)</f>
         <v>8</v>
       </c>
       <c r="K39" s="109">
@@ -5882,7 +5998,7 @@
       <c r="L39" s="13"/>
       <c r="M39" s="106"/>
       <c r="N39" s="136">
-        <f t="shared" ref="N39:N42" si="40">M39-C39</f>
+        <f t="shared" ref="N39:N42" si="44">M39-C39</f>
         <v>-46243</v>
       </c>
       <c r="O39" s="121" t="s">
@@ -5894,22 +6010,22 @@
       <c r="S39" s="131"/>
       <c r="T39" s="131"/>
       <c r="U39" s="108">
-        <f t="shared" ref="U39:U42" si="41">SUM(P39:T39)</f>
+        <f t="shared" ref="U39:U42" si="45">SUM(P39:T39)</f>
         <v>0</v>
       </c>
       <c r="V39" s="131">
-        <f t="shared" ref="V39:V42" si="42">J39-U39</f>
+        <f t="shared" ref="V39:V42" si="46">J39-U39</f>
         <v>8</v>
       </c>
       <c r="W39" s="137">
-        <f t="shared" ref="W39:W42" si="43">U39+V39</f>
+        <f t="shared" ref="W39:W42" si="47">U39+V39</f>
         <v>8</v>
       </c>
       <c r="X39" s="131" t="s">
         <v>64</v>
       </c>
       <c r="Y39" s="137">
-        <f t="shared" ref="Y39:Y42" si="44">(W39-J39)</f>
+        <f t="shared" ref="Y39:Y42" si="48">(W39-J39)</f>
         <v>0</v>
       </c>
       <c r="Z39" s="109">
@@ -5921,7 +6037,7 @@
         <v>880</v>
       </c>
       <c r="AB39" s="139">
-        <f t="shared" ref="AB39:AB43" si="45">Z39-K39</f>
+        <f t="shared" ref="AB39:AB43" si="49">Z39-K39</f>
         <v>-880</v>
       </c>
       <c r="AC39" s="6"/>
@@ -5960,7 +6076,7 @@
         <v>2</v>
       </c>
       <c r="J40" s="108">
-        <f t="shared" si="39"/>
+        <f t="shared" si="43"/>
         <v>11</v>
       </c>
       <c r="K40" s="109">
@@ -5970,7 +6086,7 @@
       <c r="L40" s="13"/>
       <c r="M40" s="106"/>
       <c r="N40" s="136">
-        <f t="shared" si="40"/>
+        <f t="shared" si="44"/>
         <v>-46240</v>
       </c>
       <c r="O40" s="121" t="s">
@@ -5982,22 +6098,22 @@
       <c r="S40" s="131"/>
       <c r="T40" s="131"/>
       <c r="U40" s="108">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="V40" s="131">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>11</v>
       </c>
       <c r="W40" s="137">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>11</v>
       </c>
       <c r="X40" s="131" t="s">
         <v>64</v>
       </c>
       <c r="Y40" s="137">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="Z40" s="109">
@@ -6009,7 +6125,7 @@
         <v>1210</v>
       </c>
       <c r="AB40" s="139">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>-1210</v>
       </c>
       <c r="AC40" s="6"/>
@@ -6046,7 +6162,7 @@
         <v>2</v>
       </c>
       <c r="J41" s="108">
-        <f t="shared" si="39"/>
+        <f t="shared" si="43"/>
         <v>10</v>
       </c>
       <c r="K41" s="109">
@@ -6056,7 +6172,7 @@
       <c r="L41" s="13"/>
       <c r="M41" s="106"/>
       <c r="N41" s="136">
-        <f t="shared" si="40"/>
+        <f t="shared" si="44"/>
         <v>-46240</v>
       </c>
       <c r="O41" s="121" t="s">
@@ -6068,22 +6184,22 @@
       <c r="S41" s="131"/>
       <c r="T41" s="131"/>
       <c r="U41" s="108">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="V41" s="131">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>10</v>
       </c>
       <c r="W41" s="137">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>10</v>
       </c>
       <c r="X41" s="131" t="s">
         <v>64</v>
       </c>
       <c r="Y41" s="137">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="Z41" s="109">
@@ -6095,7 +6211,7 @@
         <v>1100</v>
       </c>
       <c r="AB41" s="139">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>-1100</v>
       </c>
       <c r="AC41" s="6"/>
@@ -6132,7 +6248,7 @@
         <v>2</v>
       </c>
       <c r="J42" s="108">
-        <f t="shared" si="39"/>
+        <f t="shared" si="43"/>
         <v>11</v>
       </c>
       <c r="K42" s="109">
@@ -6142,7 +6258,7 @@
       <c r="L42" s="13"/>
       <c r="M42" s="106"/>
       <c r="N42" s="136">
-        <f t="shared" si="40"/>
+        <f t="shared" si="44"/>
         <v>-46243</v>
       </c>
       <c r="O42" s="116" t="s">
@@ -6154,22 +6270,22 @@
       <c r="S42" s="131"/>
       <c r="T42" s="131"/>
       <c r="U42" s="108">
-        <f t="shared" si="41"/>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="V42" s="131">
-        <f t="shared" si="42"/>
+        <f t="shared" si="46"/>
         <v>11</v>
       </c>
       <c r="W42" s="137">
-        <f t="shared" si="43"/>
+        <f t="shared" si="47"/>
         <v>11</v>
       </c>
       <c r="X42" s="131" t="s">
         <v>64</v>
       </c>
       <c r="Y42" s="137">
-        <f t="shared" si="44"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="Z42" s="109">
@@ -6181,7 +6297,7 @@
         <v>1210</v>
       </c>
       <c r="AB42" s="139">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>-1210</v>
       </c>
       <c r="AC42" s="6"/>
@@ -6209,23 +6325,23 @@
         <v>10</v>
       </c>
       <c r="F43" s="130">
-        <f t="shared" ref="F43:I43" si="46">SUM(F39:F42)</f>
+        <f t="shared" ref="F43:I43" si="50">SUM(F39:F42)</f>
         <v>7</v>
       </c>
       <c r="G43" s="130">
-        <f t="shared" si="46"/>
+        <f t="shared" si="50"/>
         <v>8</v>
       </c>
       <c r="H43" s="130">
-        <f t="shared" si="46"/>
+        <f t="shared" si="50"/>
         <v>8</v>
       </c>
       <c r="I43" s="130">
-        <f t="shared" si="46"/>
+        <f t="shared" si="50"/>
         <v>7</v>
       </c>
       <c r="J43" s="130">
-        <f t="shared" si="39"/>
+        <f t="shared" si="43"/>
         <v>40</v>
       </c>
       <c r="K43" s="71">
@@ -6245,40 +6361,40 @@
         <v>48</v>
       </c>
       <c r="P43" s="57">
-        <f t="shared" ref="P43:Y43" si="47">SUM(P39:P42)</f>
+        <f t="shared" ref="P43:Y43" si="51">SUM(P39:P42)</f>
         <v>0</v>
       </c>
       <c r="Q43" s="57">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>0</v>
       </c>
       <c r="R43" s="57">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>0</v>
       </c>
       <c r="S43" s="57">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>0</v>
       </c>
       <c r="T43" s="57">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>0</v>
       </c>
       <c r="U43" s="57">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>0</v>
       </c>
       <c r="V43" s="57">
-        <f t="shared" ref="V43" si="48">SUM(V39:V42)</f>
+        <f t="shared" ref="V43" si="52">SUM(V39:V42)</f>
         <v>40</v>
       </c>
       <c r="W43" s="57">
-        <f t="shared" ref="W43" si="49">SUM(W39:W42)</f>
+        <f t="shared" ref="W43" si="53">SUM(W39:W42)</f>
         <v>40</v>
       </c>
       <c r="X43" s="57"/>
       <c r="Y43" s="57">
-        <f t="shared" si="47"/>
+        <f t="shared" si="51"/>
         <v>0</v>
       </c>
       <c r="Z43" s="71">
@@ -6290,7 +6406,7 @@
         <v>4400</v>
       </c>
       <c r="AB43" s="71">
-        <f t="shared" si="45"/>
+        <f t="shared" si="49"/>
         <v>-4400</v>
       </c>
       <c r="AC43" s="53"/>
@@ -6360,27 +6476,27 @@
         <v>29</v>
       </c>
       <c r="E45" s="87">
-        <f t="shared" ref="E45:J45" si="50">E11+E17+E37+E43</f>
+        <f t="shared" ref="E45:J45" si="54">E11+E17+E37+E43</f>
         <v>72</v>
       </c>
       <c r="F45" s="87">
-        <f t="shared" si="50"/>
+        <f t="shared" si="54"/>
         <v>59</v>
       </c>
       <c r="G45" s="87">
-        <f t="shared" si="50"/>
+        <f t="shared" si="54"/>
         <v>60</v>
       </c>
       <c r="H45" s="87">
-        <f t="shared" si="50"/>
+        <f t="shared" si="54"/>
         <v>68</v>
       </c>
       <c r="I45" s="88">
-        <f t="shared" si="50"/>
+        <f t="shared" si="54"/>
         <v>79</v>
       </c>
       <c r="J45" s="89">
-        <f t="shared" si="50"/>
+        <f t="shared" si="54"/>
         <v>338</v>
       </c>
       <c r="K45" s="73">
@@ -6390,46 +6506,46 @@
       <c r="L45" s="27"/>
       <c r="M45" s="64">
         <f>MAX(M11,M17,M37,M43)</f>
-        <v>46213</v>
+        <v>46215</v>
       </c>
       <c r="N45" s="65">
         <f>M45-C45</f>
-        <v>-30</v>
+        <v>-28</v>
       </c>
       <c r="O45" s="26">
         <f>O37</f>
         <v>0</v>
       </c>
       <c r="P45" s="58">
-        <f t="shared" ref="P45:W45" si="51">P11+P17+P37+P43</f>
+        <f t="shared" ref="P45:W45" si="55">P11+P17+P37+P43</f>
         <v>24</v>
       </c>
       <c r="Q45" s="58">
-        <f t="shared" si="51"/>
+        <f t="shared" si="55"/>
         <v>12</v>
       </c>
       <c r="R45" s="58">
-        <f t="shared" si="51"/>
+        <f t="shared" si="55"/>
         <v>13</v>
       </c>
       <c r="S45" s="58">
-        <f t="shared" si="51"/>
+        <f t="shared" si="55"/>
         <v>16</v>
       </c>
       <c r="T45" s="58">
-        <f t="shared" si="51"/>
+        <f t="shared" si="55"/>
         <v>16</v>
       </c>
       <c r="U45" s="58">
-        <f t="shared" si="51"/>
-        <v>94</v>
+        <f t="shared" si="55"/>
+        <v>187</v>
       </c>
       <c r="V45" s="58">
-        <f t="shared" si="51"/>
-        <v>244</v>
+        <f t="shared" si="55"/>
+        <v>151</v>
       </c>
       <c r="W45" s="58">
-        <f t="shared" si="51"/>
+        <f t="shared" si="55"/>
         <v>338</v>
       </c>
       <c r="X45" s="58"/>
@@ -6439,7 +6555,7 @@
       </c>
       <c r="Z45" s="73">
         <f>Z11+Z17+Z37+Z43</f>
-        <v>10340</v>
+        <v>20570</v>
       </c>
       <c r="AA45" s="73">
         <f>AA11+AA17+AA37+AA43</f>
@@ -6447,7 +6563,7 @@
       </c>
       <c r="AB45" s="73">
         <f>Z45-K45</f>
-        <v>-26840</v>
+        <v>-16610</v>
       </c>
       <c r="AC45" s="63"/>
       <c r="AD45" s="28"/>
@@ -18325,6 +18441,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="P3:Y3"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="M18:N18"/>
     <mergeCell ref="AI17:AI20"/>
     <mergeCell ref="AE18:AH19"/>
     <mergeCell ref="B1:K1"/>
@@ -18336,25 +18457,34 @@
     <mergeCell ref="E3:J3"/>
     <mergeCell ref="M3:N3"/>
     <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="P3:Y3"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="M18:N18"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
-  <conditionalFormatting sqref="X6:X42">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Bloqué">
+  <conditionalFormatting sqref="X6:X18 X23:X42">
+    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="Bloqué">
       <formula>NOT(ISERROR(SEARCH("Bloqué",X6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",X6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="5" priority="7" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",X6)))</formula>
     </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="8" operator="containsText" text="Pas commencé">
+      <formula>NOT(ISERROR(SEARCH("Pas commencé",X6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X19:X22">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Bloqué">
+      <formula>NOT(ISERROR(SEARCH("Bloqué",X19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",X19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",X19)))</formula>
+    </cfRule>
     <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Pas commencé">
-      <formula>NOT(ISERROR(SEARCH("Pas commencé",X6)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Pas commencé",X19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>